<commit_message>
catalogue-import: keep the old printed QR numbers, new pieces start at 78
Pasting the import renumbered the sheet 7-174 in catalogue order, so the
already printed QR codes (/7 ... /77) would open the wrong pieces.

- fix-ids.xlsx: correct id + LINK per current sheet row, ready to paste
  (old pieces get their old number back; old group codes 67/70-73 open
  the first piece of their group; new pieces get 78-176)
- mia-catalogue-rows.xlsx/.csv regenerated with those ids and
  mia.nadimfoundation.org/<id> links
- qr/: codes only for the new numbers 78-176, each verified to decode
- old-printed-qr-ids.txt: the old numbering for reference

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012VHAV3HVm2aTotHZdcSemJ
</commit_message>
<xml_diff>
--- a/catalogue-import/mia-catalogue-rows.xlsx
+++ b/catalogue-import/mia-catalogue-rows.xlsx
@@ -755,7 +755,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>11612</t>
+          <t>7</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
@@ -847,7 +847,7 @@
       <c r="AR2" s="3" t="inlineStr"/>
       <c r="AS2" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q11612</t>
+          <t>https://mia.nadimfoundation.org/7</t>
         </is>
       </c>
       <c r="AT2" s="3">
@@ -876,7 +876,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>4618</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
@@ -960,7 +960,7 @@
       <c r="AR3" s="3" t="inlineStr"/>
       <c r="AS3" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4618</t>
+          <t>https://mia.nadimfoundation.org/8</t>
         </is>
       </c>
       <c r="AT3" s="3">
@@ -997,7 +997,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>3469</t>
+          <t>9</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -1081,7 +1081,7 @@
       <c r="AR4" s="3" t="inlineStr"/>
       <c r="AS4" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q3469</t>
+          <t>https://mia.nadimfoundation.org/9</t>
         </is>
       </c>
       <c r="AT4" s="3">
@@ -1102,7 +1102,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>9520</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -1194,7 +1194,7 @@
       <c r="AR5" s="3" t="inlineStr"/>
       <c r="AS5" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q9520</t>
+          <t>https://mia.nadimfoundation.org/10</t>
         </is>
       </c>
       <c r="AT5" s="3">
@@ -1223,7 +1223,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>9898</t>
+          <t>11</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -1315,7 +1315,7 @@
       <c r="AR6" s="3" t="inlineStr"/>
       <c r="AS6" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q9898</t>
+          <t>https://mia.nadimfoundation.org/11</t>
         </is>
       </c>
       <c r="AT6" s="3">
@@ -1344,7 +1344,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>4132-4133</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -1436,7 +1436,7 @@
       <c r="AR7" s="3" t="inlineStr"/>
       <c r="AS7" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4132-4133</t>
+          <t>https://mia.nadimfoundation.org/12</t>
         </is>
       </c>
       <c r="AT7" s="3">
@@ -1465,7 +1465,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>6853</t>
+          <t>13</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -1557,7 +1557,7 @@
       <c r="AR8" s="3" t="inlineStr"/>
       <c r="AS8" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q6853</t>
+          <t>https://mia.nadimfoundation.org/13</t>
         </is>
       </c>
       <c r="AT8" s="3">
@@ -1578,7 +1578,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>8367-2</t>
+          <t>14</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1670,7 +1670,7 @@
       <c r="AR9" s="3" t="inlineStr"/>
       <c r="AS9" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q8367-2</t>
+          <t>https://mia.nadimfoundation.org/14</t>
         </is>
       </c>
       <c r="AT9" s="3">
@@ -1707,7 +1707,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>16466</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1791,7 +1791,7 @@
       <c r="AR10" s="3" t="inlineStr"/>
       <c r="AS10" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q16466</t>
+          <t>https://mia.nadimfoundation.org/15</t>
         </is>
       </c>
       <c r="AT10" s="3">
@@ -1812,7 +1812,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>2112</t>
+          <t>16</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1904,7 +1904,7 @@
       <c r="AR11" s="3" t="inlineStr"/>
       <c r="AS11" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q2112</t>
+          <t>https://mia.nadimfoundation.org/16</t>
         </is>
       </c>
       <c r="AT11" s="3">
@@ -1925,7 +1925,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>14600</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -2009,7 +2009,7 @@
       <c r="AR12" s="3" t="inlineStr"/>
       <c r="AS12" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q14600</t>
+          <t>https://mia.nadimfoundation.org/17</t>
         </is>
       </c>
       <c r="AT12" s="3">
@@ -2046,7 +2046,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>16343</t>
+          <t>18</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -2130,7 +2130,7 @@
       <c r="AR13" s="3" t="inlineStr"/>
       <c r="AS13" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q16343</t>
+          <t>https://mia.nadimfoundation.org/18</t>
         </is>
       </c>
       <c r="AT13" s="3">
@@ -2167,7 +2167,7 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>14110</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -2251,7 +2251,7 @@
       <c r="AR14" s="3" t="inlineStr"/>
       <c r="AS14" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q14110</t>
+          <t>https://mia.nadimfoundation.org/19</t>
         </is>
       </c>
       <c r="AT14" s="3">
@@ -2280,7 +2280,7 @@
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>4134</t>
+          <t>20</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -2372,7 +2372,7 @@
       <c r="AR15" s="3" t="inlineStr"/>
       <c r="AS15" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4134</t>
+          <t>https://mia.nadimfoundation.org/20</t>
         </is>
       </c>
       <c r="AT15" s="3">
@@ -2393,7 +2393,7 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>3196</t>
+          <t>77</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -2487,7 +2487,7 @@
       <c r="AR16" s="3" t="inlineStr"/>
       <c r="AS16" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q3196</t>
+          <t>https://mia.nadimfoundation.org/77</t>
         </is>
       </c>
       <c r="AT16" s="3">
@@ -2516,7 +2516,7 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>9519</t>
+          <t>21</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -2608,7 +2608,7 @@
       <c r="AR17" s="3" t="inlineStr"/>
       <c r="AS17" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q9519</t>
+          <t>https://mia.nadimfoundation.org/21</t>
         </is>
       </c>
       <c r="AT17" s="3">
@@ -2637,7 +2637,7 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>8946</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -2729,7 +2729,7 @@
       <c r="AR18" s="3" t="inlineStr"/>
       <c r="AS18" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q8946</t>
+          <t>https://mia.nadimfoundation.org/22</t>
         </is>
       </c>
       <c r="AT18" s="3">
@@ -2758,7 +2758,7 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>4749</t>
+          <t>23</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -2842,7 +2842,7 @@
       <c r="AR19" s="3" t="inlineStr"/>
       <c r="AS19" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4749</t>
+          <t>https://mia.nadimfoundation.org/23</t>
         </is>
       </c>
       <c r="AT19" s="3">
@@ -2871,7 +2871,7 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>1585</t>
+          <t>24</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -2963,7 +2963,7 @@
       <c r="AR20" s="3" t="inlineStr"/>
       <c r="AS20" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q1585</t>
+          <t>https://mia.nadimfoundation.org/24</t>
         </is>
       </c>
       <c r="AT20" s="3">
@@ -2984,7 +2984,7 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>479</t>
+          <t>25</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -3076,7 +3076,7 @@
       <c r="AR21" s="3" t="inlineStr"/>
       <c r="AS21" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q479</t>
+          <t>https://mia.nadimfoundation.org/25</t>
         </is>
       </c>
       <c r="AT21" s="3">
@@ -3097,7 +3097,7 @@
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>466</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -3189,7 +3189,7 @@
       <c r="AR22" s="3" t="inlineStr"/>
       <c r="AS22" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q466</t>
+          <t>https://mia.nadimfoundation.org/26</t>
         </is>
       </c>
       <c r="AT22" s="3">
@@ -3210,7 +3210,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>467-1-2</t>
+          <t>27</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -3288,7 +3288,7 @@
       <c r="AR23" s="3" t="inlineStr"/>
       <c r="AS23" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q467-1-2</t>
+          <t>https://mia.nadimfoundation.org/27</t>
         </is>
       </c>
       <c r="AT23" s="3">
@@ -3309,7 +3309,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>1648</t>
+          <t>28</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -3401,7 +3401,7 @@
       <c r="AR24" s="3" t="inlineStr"/>
       <c r="AS24" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q1648</t>
+          <t>https://mia.nadimfoundation.org/28</t>
         </is>
       </c>
       <c r="AT24" s="3">
@@ -3422,7 +3422,7 @@
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>9748</t>
+          <t>30</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -3498,7 +3498,7 @@
       <c r="AR25" s="3" t="inlineStr"/>
       <c r="AS25" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q9748</t>
+          <t>https://mia.nadimfoundation.org/30</t>
         </is>
       </c>
       <c r="AT25" s="3">
@@ -3527,7 +3527,7 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>4140</t>
+          <t>29</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -3611,7 +3611,7 @@
       <c r="AR26" s="3" t="inlineStr"/>
       <c r="AS26" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4140</t>
+          <t>https://mia.nadimfoundation.org/29</t>
         </is>
       </c>
       <c r="AT26" s="3">
@@ -3632,7 +3632,7 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>644</t>
+          <t>31</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -3724,7 +3724,7 @@
       <c r="AR27" s="3" t="inlineStr"/>
       <c r="AS27" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q644</t>
+          <t>https://mia.nadimfoundation.org/31</t>
         </is>
       </c>
       <c r="AT27" s="3">
@@ -3745,7 +3745,7 @@
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>3132</t>
+          <t>32</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -3837,7 +3837,7 @@
       <c r="AR28" s="3" t="inlineStr"/>
       <c r="AS28" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q3132</t>
+          <t>https://mia.nadimfoundation.org/32</t>
         </is>
       </c>
       <c r="AT28" s="3">
@@ -3858,7 +3858,7 @@
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>431</t>
+          <t>33</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -3934,7 +3934,7 @@
       <c r="AR29" s="3" t="inlineStr"/>
       <c r="AS29" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q431</t>
+          <t>https://mia.nadimfoundation.org/33</t>
         </is>
       </c>
       <c r="AT29" s="3">
@@ -3955,7 +3955,7 @@
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>2972</t>
+          <t>34</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -4039,7 +4039,7 @@
       <c r="AR30" s="3" t="inlineStr"/>
       <c r="AS30" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q2972</t>
+          <t>https://mia.nadimfoundation.org/34</t>
         </is>
       </c>
       <c r="AT30" s="3">
@@ -4068,7 +4068,7 @@
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>3102</t>
+          <t>35</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -4160,7 +4160,7 @@
       <c r="AR31" s="3" t="inlineStr"/>
       <c r="AS31" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q3102</t>
+          <t>https://mia.nadimfoundation.org/35</t>
         </is>
       </c>
       <c r="AT31" s="3">
@@ -4189,7 +4189,7 @@
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>2801-4155</t>
+          <t>78</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -4283,7 +4283,7 @@
       <c r="AR32" s="3" t="inlineStr"/>
       <c r="AS32" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q2801-4155</t>
+          <t>https://mia.nadimfoundation.org/78</t>
         </is>
       </c>
       <c r="AT32" s="3">
@@ -4304,7 +4304,7 @@
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>3511</t>
+          <t>36</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -4396,7 +4396,7 @@
       <c r="AR33" s="3" t="inlineStr"/>
       <c r="AS33" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q3511</t>
+          <t>https://mia.nadimfoundation.org/36</t>
         </is>
       </c>
       <c r="AT33" s="3">
@@ -4417,7 +4417,7 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>539</t>
+          <t>37</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -4493,7 +4493,7 @@
       <c r="AR34" s="3" t="inlineStr"/>
       <c r="AS34" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q539</t>
+          <t>https://mia.nadimfoundation.org/37</t>
         </is>
       </c>
       <c r="AT34" s="3">
@@ -4514,7 +4514,7 @@
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>534</t>
+          <t>38</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -4590,7 +4590,7 @@
       <c r="AR35" s="3" t="inlineStr"/>
       <c r="AS35" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q534</t>
+          <t>https://mia.nadimfoundation.org/38</t>
         </is>
       </c>
       <c r="AT35" s="3">
@@ -4611,7 +4611,7 @@
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>485</t>
+          <t>39</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -4687,7 +4687,7 @@
       <c r="AR36" s="3" t="inlineStr"/>
       <c r="AS36" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q485</t>
+          <t>https://mia.nadimfoundation.org/39</t>
         </is>
       </c>
       <c r="AT36" s="3">
@@ -4708,7 +4708,7 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>532</t>
+          <t>40</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -4784,7 +4784,7 @@
       <c r="AR37" s="3" t="inlineStr"/>
       <c r="AS37" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q532</t>
+          <t>https://mia.nadimfoundation.org/40</t>
         </is>
       </c>
       <c r="AT37" s="3">
@@ -4805,7 +4805,7 @@
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>1048</t>
+          <t>41</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -4881,7 +4881,7 @@
       <c r="AR38" s="3" t="inlineStr"/>
       <c r="AS38" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q1048</t>
+          <t>https://mia.nadimfoundation.org/41</t>
         </is>
       </c>
       <c r="AT38" s="3">
@@ -4902,7 +4902,7 @@
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>1617</t>
+          <t>42</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -4994,7 +4994,7 @@
       <c r="AR39" s="3" t="inlineStr"/>
       <c r="AS39" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q1617</t>
+          <t>https://mia.nadimfoundation.org/42</t>
         </is>
       </c>
       <c r="AT39" s="3">
@@ -5015,7 +5015,7 @@
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>5977</t>
+          <t>45</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -5091,7 +5091,7 @@
       <c r="AR40" s="3" t="inlineStr"/>
       <c r="AS40" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q5977</t>
+          <t>https://mia.nadimfoundation.org/45</t>
         </is>
       </c>
       <c r="AT40" s="3">
@@ -5128,7 +5128,7 @@
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>445</t>
+          <t>44</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -5220,7 +5220,7 @@
       <c r="AR41" s="3" t="inlineStr"/>
       <c r="AS41" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q445</t>
+          <t>https://mia.nadimfoundation.org/44</t>
         </is>
       </c>
       <c r="AT41" s="3">
@@ -5241,7 +5241,7 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>2605</t>
+          <t>43</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -5333,7 +5333,7 @@
       <c r="AR42" s="3" t="inlineStr"/>
       <c r="AS42" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q2605</t>
+          <t>https://mia.nadimfoundation.org/43</t>
         </is>
       </c>
       <c r="AT42" s="3">
@@ -5354,7 +5354,7 @@
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>11724</t>
+          <t>46</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -5431,7 +5431,7 @@
       <c r="AR43" s="3" t="inlineStr"/>
       <c r="AS43" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q11724</t>
+          <t>https://mia.nadimfoundation.org/46</t>
         </is>
       </c>
       <c r="AT43" s="3">
@@ -5468,7 +5468,7 @@
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>11718</t>
+          <t>47</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -5544,7 +5544,7 @@
       <c r="AR44" s="3" t="inlineStr"/>
       <c r="AS44" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q11718</t>
+          <t>https://mia.nadimfoundation.org/47</t>
         </is>
       </c>
       <c r="AT44" s="3">
@@ -5573,7 +5573,7 @@
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
-          <t>11721</t>
+          <t>48</t>
         </is>
       </c>
       <c r="B45" s="3" t="inlineStr">
@@ -5651,7 +5651,7 @@
       <c r="AR45" s="3" t="inlineStr"/>
       <c r="AS45" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q11721</t>
+          <t>https://mia.nadimfoundation.org/48</t>
         </is>
       </c>
       <c r="AT45" s="3">
@@ -5688,7 +5688,7 @@
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>9526</t>
+          <t>49</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -5772,7 +5772,7 @@
       <c r="AR46" s="3" t="inlineStr"/>
       <c r="AS46" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q9526</t>
+          <t>https://mia.nadimfoundation.org/49</t>
         </is>
       </c>
       <c r="AT46" s="3">
@@ -5809,7 +5809,7 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>3555-1-5</t>
+          <t>50</t>
         </is>
       </c>
       <c r="B47" s="3" t="inlineStr">
@@ -5903,7 +5903,7 @@
       <c r="AR47" s="3" t="inlineStr"/>
       <c r="AS47" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q3555-1-5</t>
+          <t>https://mia.nadimfoundation.org/50</t>
         </is>
       </c>
       <c r="AT47" s="3">
@@ -5932,7 +5932,7 @@
     <row r="48">
       <c r="A48" s="3" t="inlineStr">
         <is>
-          <t>11747</t>
+          <t>51</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
@@ -6024,7 +6024,7 @@
       <c r="AR48" s="3" t="inlineStr"/>
       <c r="AS48" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q11747</t>
+          <t>https://mia.nadimfoundation.org/51</t>
         </is>
       </c>
       <c r="AT48" s="3">
@@ -6045,7 +6045,7 @@
     <row r="49">
       <c r="A49" s="3" t="inlineStr">
         <is>
-          <t>403-405</t>
+          <t>52</t>
         </is>
       </c>
       <c r="B49" s="3" t="inlineStr">
@@ -6139,7 +6139,7 @@
       <c r="AR49" s="3" t="inlineStr"/>
       <c r="AS49" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q403-405</t>
+          <t>https://mia.nadimfoundation.org/52</t>
         </is>
       </c>
       <c r="AT49" s="3">
@@ -6160,7 +6160,7 @@
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>621-1-2</t>
+          <t>53</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -6238,7 +6238,7 @@
       <c r="AR50" s="3" t="inlineStr"/>
       <c r="AS50" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q621-1-2</t>
+          <t>https://mia.nadimfoundation.org/53</t>
         </is>
       </c>
       <c r="AT50" s="3">
@@ -6259,7 +6259,7 @@
     <row r="51">
       <c r="A51" s="3" t="inlineStr">
         <is>
-          <t>550</t>
+          <t>54</t>
         </is>
       </c>
       <c r="B51" s="3" t="inlineStr">
@@ -6335,7 +6335,7 @@
       <c r="AR51" s="3" t="inlineStr"/>
       <c r="AS51" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q550</t>
+          <t>https://mia.nadimfoundation.org/54</t>
         </is>
       </c>
       <c r="AT51" s="3">
@@ -6356,7 +6356,7 @@
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>528</t>
+          <t>55</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
@@ -6432,7 +6432,7 @@
       <c r="AR52" s="3" t="inlineStr"/>
       <c r="AS52" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q528</t>
+          <t>https://mia.nadimfoundation.org/55</t>
         </is>
       </c>
       <c r="AT52" s="3">
@@ -6453,7 +6453,7 @@
     <row r="53">
       <c r="A53" s="3" t="inlineStr">
         <is>
-          <t>505</t>
+          <t>56</t>
         </is>
       </c>
       <c r="B53" s="3" t="inlineStr">
@@ -6537,7 +6537,7 @@
       <c r="AR53" s="3" t="inlineStr"/>
       <c r="AS53" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q505</t>
+          <t>https://mia.nadimfoundation.org/56</t>
         </is>
       </c>
       <c r="AT53" s="3">
@@ -6558,7 +6558,7 @@
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>3512</t>
+          <t>57</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
@@ -6650,7 +6650,7 @@
       <c r="AR54" s="3" t="inlineStr"/>
       <c r="AS54" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q3512</t>
+          <t>https://mia.nadimfoundation.org/57</t>
         </is>
       </c>
       <c r="AT54" s="3">
@@ -6679,7 +6679,7 @@
     <row r="55">
       <c r="A55" s="3" t="inlineStr">
         <is>
-          <t>4392</t>
+          <t>58</t>
         </is>
       </c>
       <c r="B55" s="3" t="inlineStr">
@@ -6771,7 +6771,7 @@
       <c r="AR55" s="3" t="inlineStr"/>
       <c r="AS55" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4392</t>
+          <t>https://mia.nadimfoundation.org/58</t>
         </is>
       </c>
       <c r="AT55" s="3">
@@ -6800,7 +6800,7 @@
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>612</t>
+          <t>59</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
@@ -6876,7 +6876,7 @@
       <c r="AR56" s="3" t="inlineStr"/>
       <c r="AS56" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q612</t>
+          <t>https://mia.nadimfoundation.org/59</t>
         </is>
       </c>
       <c r="AT56" s="3">
@@ -6897,7 +6897,7 @@
     <row r="57">
       <c r="A57" s="3" t="inlineStr">
         <is>
-          <t>11641</t>
+          <t>60</t>
         </is>
       </c>
       <c r="B57" s="3" t="inlineStr">
@@ -6981,7 +6981,7 @@
       <c r="AR57" s="3" t="inlineStr"/>
       <c r="AS57" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q11641</t>
+          <t>https://mia.nadimfoundation.org/60</t>
         </is>
       </c>
       <c r="AT57" s="3">
@@ -7010,7 +7010,7 @@
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>1421</t>
+          <t>61</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
@@ -7086,7 +7086,7 @@
       <c r="AR58" s="3" t="inlineStr"/>
       <c r="AS58" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q1421</t>
+          <t>https://mia.nadimfoundation.org/61</t>
         </is>
       </c>
       <c r="AT58" s="3">
@@ -7107,7 +7107,7 @@
     <row r="59">
       <c r="A59" s="3" t="inlineStr">
         <is>
-          <t>6857</t>
+          <t>62</t>
         </is>
       </c>
       <c r="B59" s="3" t="inlineStr">
@@ -7191,7 +7191,7 @@
       <c r="AR59" s="3" t="inlineStr"/>
       <c r="AS59" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q6857</t>
+          <t>https://mia.nadimfoundation.org/62</t>
         </is>
       </c>
       <c r="AT59" s="3">
@@ -7220,7 +7220,7 @@
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>2602</t>
+          <t>63</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
@@ -7304,7 +7304,7 @@
       <c r="AR60" s="3" t="inlineStr"/>
       <c r="AS60" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q2602</t>
+          <t>https://mia.nadimfoundation.org/63</t>
         </is>
       </c>
       <c r="AT60" s="3">
@@ -7333,7 +7333,7 @@
     <row r="61">
       <c r="A61" s="3" t="inlineStr">
         <is>
-          <t>3484</t>
+          <t>64</t>
         </is>
       </c>
       <c r="B61" s="3" t="inlineStr">
@@ -7425,7 +7425,7 @@
       <c r="AR61" s="3" t="inlineStr"/>
       <c r="AS61" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q3484</t>
+          <t>https://mia.nadimfoundation.org/64</t>
         </is>
       </c>
       <c r="AT61" s="3">
@@ -7454,7 +7454,7 @@
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>3485</t>
+          <t>65</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
@@ -7546,7 +7546,7 @@
       <c r="AR62" s="3" t="inlineStr"/>
       <c r="AS62" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q3485</t>
+          <t>https://mia.nadimfoundation.org/65</t>
         </is>
       </c>
       <c r="AT62" s="3">
@@ -7567,7 +7567,7 @@
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>4144</t>
+          <t>66</t>
         </is>
       </c>
       <c r="B63" s="3" t="inlineStr">
@@ -7653,7 +7653,7 @@
       <c r="AR63" s="3" t="inlineStr"/>
       <c r="AS63" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4144</t>
+          <t>https://mia.nadimfoundation.org/66</t>
         </is>
       </c>
       <c r="AT63" s="3">
@@ -7674,7 +7674,7 @@
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>6120-6</t>
+          <t>68</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
@@ -7750,7 +7750,7 @@
       <c r="AR64" s="3" t="inlineStr"/>
       <c r="AS64" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q6120-6</t>
+          <t>https://mia.nadimfoundation.org/68</t>
         </is>
       </c>
       <c r="AT64" s="3">
@@ -7787,7 +7787,7 @@
     <row r="65">
       <c r="A65" s="3" t="inlineStr">
         <is>
-          <t>6120-4</t>
+          <t>67</t>
         </is>
       </c>
       <c r="B65" s="3" t="inlineStr">
@@ -7863,7 +7863,7 @@
       <c r="AR65" s="3" t="inlineStr"/>
       <c r="AS65" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q6120-4</t>
+          <t>https://mia.nadimfoundation.org/67</t>
         </is>
       </c>
       <c r="AT65" s="3">
@@ -7900,7 +7900,7 @@
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>6120-5</t>
+          <t>79</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
@@ -7976,7 +7976,7 @@
       <c r="AR66" s="3" t="inlineStr"/>
       <c r="AS66" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q6120-5</t>
+          <t>https://mia.nadimfoundation.org/79</t>
         </is>
       </c>
       <c r="AT66" s="3">
@@ -8013,7 +8013,7 @@
     <row r="67">
       <c r="A67" s="3" t="inlineStr">
         <is>
-          <t>18858-1</t>
+          <t>80</t>
         </is>
       </c>
       <c r="B67" s="3" t="inlineStr">
@@ -8089,7 +8089,7 @@
       <c r="AR67" s="3" t="inlineStr"/>
       <c r="AS67" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18858-1</t>
+          <t>https://mia.nadimfoundation.org/80</t>
         </is>
       </c>
       <c r="AT67" s="3">
@@ -8126,7 +8126,7 @@
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>18858-2</t>
+          <t>81</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
@@ -8202,7 +8202,7 @@
       <c r="AR68" s="3" t="inlineStr"/>
       <c r="AS68" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18858-2</t>
+          <t>https://mia.nadimfoundation.org/81</t>
         </is>
       </c>
       <c r="AT68" s="3">
@@ -8243,7 +8243,7 @@
     <row r="69">
       <c r="A69" s="3" t="inlineStr">
         <is>
-          <t>18858-3</t>
+          <t>82</t>
         </is>
       </c>
       <c r="B69" s="3" t="inlineStr">
@@ -8319,7 +8319,7 @@
       <c r="AR69" s="3" t="inlineStr"/>
       <c r="AS69" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18858-3</t>
+          <t>https://mia.nadimfoundation.org/82</t>
         </is>
       </c>
       <c r="AT69" s="3">
@@ -8360,7 +8360,7 @@
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>18858-4</t>
+          <t>83</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
@@ -8436,7 +8436,7 @@
       <c r="AR70" s="3" t="inlineStr"/>
       <c r="AS70" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18858-4</t>
+          <t>https://mia.nadimfoundation.org/83</t>
         </is>
       </c>
       <c r="AT70" s="3">
@@ -8477,7 +8477,7 @@
     <row r="71">
       <c r="A71" s="3" t="inlineStr">
         <is>
-          <t>18858-6</t>
+          <t>84</t>
         </is>
       </c>
       <c r="B71" s="3" t="inlineStr">
@@ -8553,7 +8553,7 @@
       <c r="AR71" s="3" t="inlineStr"/>
       <c r="AS71" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18858-6</t>
+          <t>https://mia.nadimfoundation.org/84</t>
         </is>
       </c>
       <c r="AT71" s="3">
@@ -8594,7 +8594,7 @@
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>18858-7</t>
+          <t>85</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
@@ -8670,7 +8670,7 @@
       <c r="AR72" s="3" t="inlineStr"/>
       <c r="AS72" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18858-7</t>
+          <t>https://mia.nadimfoundation.org/85</t>
         </is>
       </c>
       <c r="AT72" s="3">
@@ -8711,7 +8711,7 @@
     <row r="73">
       <c r="A73" s="3" t="inlineStr">
         <is>
-          <t>18858-8</t>
+          <t>86</t>
         </is>
       </c>
       <c r="B73" s="3" t="inlineStr">
@@ -8787,7 +8787,7 @@
       <c r="AR73" s="3" t="inlineStr"/>
       <c r="AS73" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18858-8</t>
+          <t>https://mia.nadimfoundation.org/86</t>
         </is>
       </c>
       <c r="AT73" s="3">
@@ -8828,7 +8828,7 @@
     <row r="74">
       <c r="A74" s="3" t="inlineStr">
         <is>
-          <t>21619-1</t>
+          <t>87</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
@@ -8904,7 +8904,7 @@
       <c r="AR74" s="3" t="inlineStr"/>
       <c r="AS74" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q21619-1</t>
+          <t>https://mia.nadimfoundation.org/87</t>
         </is>
       </c>
       <c r="AT74" s="3">
@@ -8937,7 +8937,7 @@
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
-          <t>21619-2</t>
+          <t>88</t>
         </is>
       </c>
       <c r="B75" s="3" t="inlineStr">
@@ -9013,7 +9013,7 @@
       <c r="AR75" s="3" t="inlineStr"/>
       <c r="AS75" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q21619-2</t>
+          <t>https://mia.nadimfoundation.org/88</t>
         </is>
       </c>
       <c r="AT75" s="3">
@@ -9046,7 +9046,7 @@
     <row r="76">
       <c r="A76" s="3" t="inlineStr">
         <is>
-          <t>21619-4</t>
+          <t>89</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
@@ -9122,7 +9122,7 @@
       <c r="AR76" s="3" t="inlineStr"/>
       <c r="AS76" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q21619-4</t>
+          <t>https://mia.nadimfoundation.org/89</t>
         </is>
       </c>
       <c r="AT76" s="3">
@@ -9155,7 +9155,7 @@
     <row r="77">
       <c r="A77" s="3" t="inlineStr">
         <is>
-          <t>7054</t>
+          <t>69</t>
         </is>
       </c>
       <c r="B77" s="3" t="inlineStr">
@@ -9231,7 +9231,7 @@
       <c r="AR77" s="3" t="inlineStr"/>
       <c r="AS77" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q7054</t>
+          <t>https://mia.nadimfoundation.org/69</t>
         </is>
       </c>
       <c r="AT77" s="3">
@@ -9252,7 +9252,7 @@
     <row r="78">
       <c r="A78" s="3" t="inlineStr">
         <is>
-          <t>18860-1</t>
+          <t>70</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
@@ -9328,7 +9328,7 @@
       <c r="AR78" s="3" t="inlineStr"/>
       <c r="AS78" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18860-1</t>
+          <t>https://mia.nadimfoundation.org/70</t>
         </is>
       </c>
       <c r="AT78" s="3">
@@ -9349,7 +9349,7 @@
     <row r="79">
       <c r="A79" s="3" t="inlineStr">
         <is>
-          <t>21618-1</t>
+          <t>90</t>
         </is>
       </c>
       <c r="B79" s="3" t="inlineStr">
@@ -9425,7 +9425,7 @@
       <c r="AR79" s="3" t="inlineStr"/>
       <c r="AS79" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q21618-1</t>
+          <t>https://mia.nadimfoundation.org/90</t>
         </is>
       </c>
       <c r="AT79" s="3">
@@ -9454,7 +9454,7 @@
     <row r="80">
       <c r="A80" s="3" t="inlineStr">
         <is>
-          <t>2588</t>
+          <t>71</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
@@ -9530,7 +9530,7 @@
       <c r="AR80" s="3" t="inlineStr"/>
       <c r="AS80" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q2588</t>
+          <t>https://mia.nadimfoundation.org/71</t>
         </is>
       </c>
       <c r="AT80" s="3">
@@ -9559,7 +9559,7 @@
     <row r="81">
       <c r="A81" s="3" t="inlineStr">
         <is>
-          <t>3883</t>
+          <t>91</t>
         </is>
       </c>
       <c r="B81" s="3" t="inlineStr">
@@ -9635,7 +9635,7 @@
       <c r="AR81" s="3" t="inlineStr"/>
       <c r="AS81" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q3883</t>
+          <t>https://mia.nadimfoundation.org/91</t>
         </is>
       </c>
       <c r="AT81" s="3">
@@ -9664,7 +9664,7 @@
     <row r="82">
       <c r="A82" s="3" t="inlineStr">
         <is>
-          <t>4920</t>
+          <t>92</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
@@ -9748,7 +9748,7 @@
       <c r="AR82" s="3" t="inlineStr"/>
       <c r="AS82" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4920</t>
+          <t>https://mia.nadimfoundation.org/92</t>
         </is>
       </c>
       <c r="AT82" s="3">
@@ -9769,7 +9769,7 @@
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
-          <t>4922</t>
+          <t>93</t>
         </is>
       </c>
       <c r="B83" s="3" t="inlineStr">
@@ -9853,7 +9853,7 @@
       <c r="AR83" s="3" t="inlineStr"/>
       <c r="AS83" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4922</t>
+          <t>https://mia.nadimfoundation.org/93</t>
         </is>
       </c>
       <c r="AT83" s="3">
@@ -9874,7 +9874,7 @@
     <row r="84">
       <c r="A84" s="3" t="inlineStr">
         <is>
-          <t>4923</t>
+          <t>94</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
@@ -9958,7 +9958,7 @@
       <c r="AR84" s="3" t="inlineStr"/>
       <c r="AS84" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4923</t>
+          <t>https://mia.nadimfoundation.org/94</t>
         </is>
       </c>
       <c r="AT84" s="3">
@@ -9979,7 +9979,7 @@
     <row r="85">
       <c r="A85" s="3" t="inlineStr">
         <is>
-          <t>4927</t>
+          <t>95</t>
         </is>
       </c>
       <c r="B85" s="3" t="inlineStr">
@@ -10063,7 +10063,7 @@
       <c r="AR85" s="3" t="inlineStr"/>
       <c r="AS85" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4927</t>
+          <t>https://mia.nadimfoundation.org/95</t>
         </is>
       </c>
       <c r="AT85" s="3">
@@ -10084,7 +10084,7 @@
     <row r="86">
       <c r="A86" s="3" t="inlineStr">
         <is>
-          <t>4929</t>
+          <t>96</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
@@ -10168,7 +10168,7 @@
       <c r="AR86" s="3" t="inlineStr"/>
       <c r="AS86" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4929</t>
+          <t>https://mia.nadimfoundation.org/96</t>
         </is>
       </c>
       <c r="AT86" s="3">
@@ -10189,7 +10189,7 @@
     <row r="87">
       <c r="A87" s="3" t="inlineStr">
         <is>
-          <t>4930</t>
+          <t>97</t>
         </is>
       </c>
       <c r="B87" s="3" t="inlineStr">
@@ -10281,7 +10281,7 @@
       <c r="AR87" s="3" t="inlineStr"/>
       <c r="AS87" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4930</t>
+          <t>https://mia.nadimfoundation.org/97</t>
         </is>
       </c>
       <c r="AT87" s="3">
@@ -10302,7 +10302,7 @@
     <row r="88">
       <c r="A88" s="3" t="inlineStr">
         <is>
-          <t>4933</t>
+          <t>98</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
@@ -10386,7 +10386,7 @@
       <c r="AR88" s="3" t="inlineStr"/>
       <c r="AS88" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4933</t>
+          <t>https://mia.nadimfoundation.org/98</t>
         </is>
       </c>
       <c r="AT88" s="3">
@@ -10407,7 +10407,7 @@
     <row r="89">
       <c r="A89" s="3" t="inlineStr">
         <is>
-          <t>4934</t>
+          <t>99</t>
         </is>
       </c>
       <c r="B89" s="3" t="inlineStr">
@@ -10491,7 +10491,7 @@
       <c r="AR89" s="3" t="inlineStr"/>
       <c r="AS89" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4934</t>
+          <t>https://mia.nadimfoundation.org/99</t>
         </is>
       </c>
       <c r="AT89" s="3">
@@ -10512,7 +10512,7 @@
     <row r="90">
       <c r="A90" s="3" t="inlineStr">
         <is>
-          <t>4935</t>
+          <t>100</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
@@ -10596,7 +10596,7 @@
       <c r="AR90" s="3" t="inlineStr"/>
       <c r="AS90" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4935</t>
+          <t>https://mia.nadimfoundation.org/100</t>
         </is>
       </c>
       <c r="AT90" s="3">
@@ -10617,7 +10617,7 @@
     <row r="91">
       <c r="A91" s="3" t="inlineStr">
         <is>
-          <t>4936</t>
+          <t>101</t>
         </is>
       </c>
       <c r="B91" s="3" t="inlineStr">
@@ -10701,7 +10701,7 @@
       <c r="AR91" s="3" t="inlineStr"/>
       <c r="AS91" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4936</t>
+          <t>https://mia.nadimfoundation.org/101</t>
         </is>
       </c>
       <c r="AT91" s="3">
@@ -10722,7 +10722,7 @@
     <row r="92">
       <c r="A92" s="3" t="inlineStr">
         <is>
-          <t>4937</t>
+          <t>102</t>
         </is>
       </c>
       <c r="B92" s="3" t="inlineStr">
@@ -10806,7 +10806,7 @@
       <c r="AR92" s="3" t="inlineStr"/>
       <c r="AS92" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4937</t>
+          <t>https://mia.nadimfoundation.org/102</t>
         </is>
       </c>
       <c r="AT92" s="3">
@@ -10827,7 +10827,7 @@
     <row r="93">
       <c r="A93" s="3" t="inlineStr">
         <is>
-          <t>6621-2</t>
+          <t>103</t>
         </is>
       </c>
       <c r="B93" s="3" t="inlineStr">
@@ -10903,7 +10903,7 @@
       <c r="AR93" s="3" t="inlineStr"/>
       <c r="AS93" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q6621-2</t>
+          <t>https://mia.nadimfoundation.org/103</t>
         </is>
       </c>
       <c r="AT93" s="3">
@@ -10940,7 +10940,7 @@
     <row r="94">
       <c r="A94" s="3" t="inlineStr">
         <is>
-          <t>8323</t>
+          <t>104</t>
         </is>
       </c>
       <c r="B94" s="3" t="inlineStr">
@@ -11016,7 +11016,7 @@
       <c r="AR94" s="3" t="inlineStr"/>
       <c r="AS94" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q8323</t>
+          <t>https://mia.nadimfoundation.org/104</t>
         </is>
       </c>
       <c r="AT94" s="3">
@@ -11053,7 +11053,7 @@
     <row r="95">
       <c r="A95" s="3" t="inlineStr">
         <is>
-          <t>9273</t>
+          <t>105</t>
         </is>
       </c>
       <c r="B95" s="3" t="inlineStr">
@@ -11129,7 +11129,7 @@
       <c r="AR95" s="3" t="inlineStr"/>
       <c r="AS95" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q9273</t>
+          <t>https://mia.nadimfoundation.org/105</t>
         </is>
       </c>
       <c r="AT95" s="3">
@@ -11158,7 +11158,7 @@
     <row r="96">
       <c r="A96" s="3" t="inlineStr">
         <is>
-          <t>9274</t>
+          <t>106</t>
         </is>
       </c>
       <c r="B96" s="3" t="inlineStr">
@@ -11234,7 +11234,7 @@
       <c r="AR96" s="3" t="inlineStr"/>
       <c r="AS96" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q9274</t>
+          <t>https://mia.nadimfoundation.org/106</t>
         </is>
       </c>
       <c r="AT96" s="3">
@@ -11263,7 +11263,7 @@
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>14766</t>
+          <t>107</t>
         </is>
       </c>
       <c r="B97" s="3" t="inlineStr">
@@ -11347,7 +11347,7 @@
       <c r="AR97" s="3" t="inlineStr"/>
       <c r="AS97" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q14766</t>
+          <t>https://mia.nadimfoundation.org/107</t>
         </is>
       </c>
       <c r="AT97" s="3">
@@ -11376,7 +11376,7 @@
     <row r="98">
       <c r="A98" s="3" t="inlineStr">
         <is>
-          <t>18764-1</t>
+          <t>108</t>
         </is>
       </c>
       <c r="B98" s="3" t="inlineStr">
@@ -11452,7 +11452,7 @@
       <c r="AR98" s="3" t="inlineStr"/>
       <c r="AS98" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18764-1</t>
+          <t>https://mia.nadimfoundation.org/108</t>
         </is>
       </c>
       <c r="AT98" s="3">
@@ -11489,7 +11489,7 @@
     <row r="99">
       <c r="A99" s="3" t="inlineStr">
         <is>
-          <t>18764-2</t>
+          <t>109</t>
         </is>
       </c>
       <c r="B99" s="3" t="inlineStr">
@@ -11565,7 +11565,7 @@
       <c r="AR99" s="3" t="inlineStr"/>
       <c r="AS99" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18764-2</t>
+          <t>https://mia.nadimfoundation.org/109</t>
         </is>
       </c>
       <c r="AT99" s="3">
@@ -11602,7 +11602,7 @@
     <row r="100">
       <c r="A100" s="3" t="inlineStr">
         <is>
-          <t>18764-3</t>
+          <t>110</t>
         </is>
       </c>
       <c r="B100" s="3" t="inlineStr">
@@ -11678,7 +11678,7 @@
       <c r="AR100" s="3" t="inlineStr"/>
       <c r="AS100" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18764-3</t>
+          <t>https://mia.nadimfoundation.org/110</t>
         </is>
       </c>
       <c r="AT100" s="3">
@@ -11715,7 +11715,7 @@
     <row r="101">
       <c r="A101" s="3" t="inlineStr">
         <is>
-          <t>18764-8</t>
+          <t>111</t>
         </is>
       </c>
       <c r="B101" s="3" t="inlineStr">
@@ -11791,7 +11791,7 @@
       <c r="AR101" s="3" t="inlineStr"/>
       <c r="AS101" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18764-8</t>
+          <t>https://mia.nadimfoundation.org/111</t>
         </is>
       </c>
       <c r="AT101" s="3">
@@ -11828,7 +11828,7 @@
     <row r="102">
       <c r="A102" s="3" t="inlineStr">
         <is>
-          <t>19400-3</t>
+          <t>112</t>
         </is>
       </c>
       <c r="B102" s="3" t="inlineStr">
@@ -11904,7 +11904,7 @@
       <c r="AR102" s="3" t="inlineStr"/>
       <c r="AS102" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q19400-3</t>
+          <t>https://mia.nadimfoundation.org/112</t>
         </is>
       </c>
       <c r="AT102" s="3">
@@ -11941,7 +11941,7 @@
     <row r="103">
       <c r="A103" s="3" t="inlineStr">
         <is>
-          <t>20660-1</t>
+          <t>113</t>
         </is>
       </c>
       <c r="B103" s="3" t="inlineStr">
@@ -12017,7 +12017,7 @@
       <c r="AR103" s="3" t="inlineStr"/>
       <c r="AS103" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q20660-1</t>
+          <t>https://mia.nadimfoundation.org/113</t>
         </is>
       </c>
       <c r="AT103" s="3">
@@ -12046,7 +12046,7 @@
     <row r="104">
       <c r="A104" s="3" t="inlineStr">
         <is>
-          <t>20660-2</t>
+          <t>114</t>
         </is>
       </c>
       <c r="B104" s="3" t="inlineStr">
@@ -12122,7 +12122,7 @@
       <c r="AR104" s="3" t="inlineStr"/>
       <c r="AS104" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q20660-2</t>
+          <t>https://mia.nadimfoundation.org/114</t>
         </is>
       </c>
       <c r="AT104" s="3">
@@ -12151,7 +12151,7 @@
     <row r="105">
       <c r="A105" s="3" t="inlineStr">
         <is>
-          <t>21520-1</t>
+          <t>115</t>
         </is>
       </c>
       <c r="B105" s="3" t="inlineStr">
@@ -12227,7 +12227,7 @@
       <c r="AR105" s="3" t="inlineStr"/>
       <c r="AS105" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q21520-1</t>
+          <t>https://mia.nadimfoundation.org/115</t>
         </is>
       </c>
       <c r="AT105" s="3">
@@ -12256,7 +12256,7 @@
     <row r="106">
       <c r="A106" s="3" t="inlineStr">
         <is>
-          <t>21520-2</t>
+          <t>116</t>
         </is>
       </c>
       <c r="B106" s="3" t="inlineStr">
@@ -12332,7 +12332,7 @@
       <c r="AR106" s="3" t="inlineStr"/>
       <c r="AS106" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q21520-2</t>
+          <t>https://mia.nadimfoundation.org/116</t>
         </is>
       </c>
       <c r="AT106" s="3">
@@ -12361,7 +12361,7 @@
     <row r="107">
       <c r="A107" s="3" t="inlineStr">
         <is>
-          <t>21520-3</t>
+          <t>117</t>
         </is>
       </c>
       <c r="B107" s="3" t="inlineStr">
@@ -12437,7 +12437,7 @@
       <c r="AR107" s="3" t="inlineStr"/>
       <c r="AS107" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q21520-3</t>
+          <t>https://mia.nadimfoundation.org/117</t>
         </is>
       </c>
       <c r="AT107" s="3">
@@ -12466,7 +12466,7 @@
     <row r="108">
       <c r="A108" s="3" t="inlineStr">
         <is>
-          <t>21520-4</t>
+          <t>118</t>
         </is>
       </c>
       <c r="B108" s="3" t="inlineStr">
@@ -12542,7 +12542,7 @@
       <c r="AR108" s="3" t="inlineStr"/>
       <c r="AS108" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q21520-4</t>
+          <t>https://mia.nadimfoundation.org/118</t>
         </is>
       </c>
       <c r="AT108" s="3">
@@ -12571,7 +12571,7 @@
     <row r="109">
       <c r="A109" s="3" t="inlineStr">
         <is>
-          <t>21520-5</t>
+          <t>119</t>
         </is>
       </c>
       <c r="B109" s="3" t="inlineStr">
@@ -12647,7 +12647,7 @@
       <c r="AR109" s="3" t="inlineStr"/>
       <c r="AS109" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q21520-5</t>
+          <t>https://mia.nadimfoundation.org/119</t>
         </is>
       </c>
       <c r="AT109" s="3">
@@ -12676,7 +12676,7 @@
     <row r="110">
       <c r="A110" s="3" t="inlineStr">
         <is>
-          <t>21520-6</t>
+          <t>120</t>
         </is>
       </c>
       <c r="B110" s="3" t="inlineStr">
@@ -12752,7 +12752,7 @@
       <c r="AR110" s="3" t="inlineStr"/>
       <c r="AS110" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q21520-6</t>
+          <t>https://mia.nadimfoundation.org/120</t>
         </is>
       </c>
       <c r="AT110" s="3">
@@ -12781,7 +12781,7 @@
     <row r="111">
       <c r="A111" s="3" t="inlineStr">
         <is>
-          <t>21618-2</t>
+          <t>121</t>
         </is>
       </c>
       <c r="B111" s="3" t="inlineStr">
@@ -12857,7 +12857,7 @@
       <c r="AR111" s="3" t="inlineStr"/>
       <c r="AS111" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q21618-2</t>
+          <t>https://mia.nadimfoundation.org/121</t>
         </is>
       </c>
       <c r="AT111" s="3">
@@ -12878,7 +12878,7 @@
     <row r="112">
       <c r="A112" s="3" t="inlineStr">
         <is>
-          <t>23497</t>
+          <t>122</t>
         </is>
       </c>
       <c r="B112" s="3" t="inlineStr">
@@ -12962,7 +12962,7 @@
       <c r="AR112" s="3" t="inlineStr"/>
       <c r="AS112" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q23497</t>
+          <t>https://mia.nadimfoundation.org/122</t>
         </is>
       </c>
       <c r="AT112" s="3">
@@ -12991,7 +12991,7 @@
     <row r="113">
       <c r="A113" s="3" t="inlineStr">
         <is>
-          <t>4926</t>
+          <t>72</t>
         </is>
       </c>
       <c r="B113" s="3" t="inlineStr">
@@ -13083,7 +13083,7 @@
       <c r="AR113" s="3" t="inlineStr"/>
       <c r="AS113" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4926</t>
+          <t>https://mia.nadimfoundation.org/72</t>
         </is>
       </c>
       <c r="AT113" s="3">
@@ -13104,7 +13104,7 @@
     <row r="114">
       <c r="A114" s="3" t="inlineStr">
         <is>
-          <t>8199</t>
+          <t>123</t>
         </is>
       </c>
       <c r="B114" s="3" t="inlineStr">
@@ -13188,7 +13188,7 @@
       <c r="AR114" s="3" t="inlineStr"/>
       <c r="AS114" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q8199</t>
+          <t>https://mia.nadimfoundation.org/123</t>
         </is>
       </c>
       <c r="AT114" s="3">
@@ -13225,7 +13225,7 @@
     <row r="115">
       <c r="A115" s="3" t="inlineStr">
         <is>
-          <t>18762-1</t>
+          <t>124</t>
         </is>
       </c>
       <c r="B115" s="3" t="inlineStr">
@@ -13309,7 +13309,7 @@
       <c r="AR115" s="3" t="inlineStr"/>
       <c r="AS115" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18762-1</t>
+          <t>https://mia.nadimfoundation.org/124</t>
         </is>
       </c>
       <c r="AT115" s="3">
@@ -13346,7 +13346,7 @@
     <row r="116">
       <c r="A116" s="3" t="inlineStr">
         <is>
-          <t>18762-2</t>
+          <t>125</t>
         </is>
       </c>
       <c r="B116" s="3" t="inlineStr">
@@ -13430,7 +13430,7 @@
       <c r="AR116" s="3" t="inlineStr"/>
       <c r="AS116" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18762-2</t>
+          <t>https://mia.nadimfoundation.org/125</t>
         </is>
       </c>
       <c r="AT116" s="3">
@@ -13467,7 +13467,7 @@
     <row r="117">
       <c r="A117" s="3" t="inlineStr">
         <is>
-          <t>18765-7</t>
+          <t>126</t>
         </is>
       </c>
       <c r="B117" s="3" t="inlineStr">
@@ -13543,7 +13543,7 @@
       <c r="AR117" s="3" t="inlineStr"/>
       <c r="AS117" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18765-7</t>
+          <t>https://mia.nadimfoundation.org/126</t>
         </is>
       </c>
       <c r="AT117" s="3">
@@ -13580,7 +13580,7 @@
     <row r="118">
       <c r="A118" s="3" t="inlineStr">
         <is>
-          <t>18766-2</t>
+          <t>127</t>
         </is>
       </c>
       <c r="B118" s="3" t="inlineStr">
@@ -13656,7 +13656,7 @@
       <c r="AR118" s="3" t="inlineStr"/>
       <c r="AS118" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18766-2</t>
+          <t>https://mia.nadimfoundation.org/127</t>
         </is>
       </c>
       <c r="AT118" s="3">
@@ -13693,7 +13693,7 @@
     <row r="119">
       <c r="A119" s="3" t="inlineStr">
         <is>
-          <t>4931</t>
+          <t>128</t>
         </is>
       </c>
       <c r="B119" s="3" t="inlineStr">
@@ -13781,7 +13781,7 @@
       <c r="AR119" s="3" t="inlineStr"/>
       <c r="AS119" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4931</t>
+          <t>https://mia.nadimfoundation.org/128</t>
         </is>
       </c>
       <c r="AT119" s="3">
@@ -13802,7 +13802,7 @@
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
         <is>
-          <t>18766-1</t>
+          <t>129</t>
         </is>
       </c>
       <c r="B120" s="3" t="inlineStr">
@@ -13878,7 +13878,7 @@
       <c r="AR120" s="3" t="inlineStr"/>
       <c r="AS120" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18766-1</t>
+          <t>https://mia.nadimfoundation.org/129</t>
         </is>
       </c>
       <c r="AT120" s="3">
@@ -13919,7 +13919,7 @@
     <row r="121">
       <c r="A121" s="3" t="inlineStr">
         <is>
-          <t>18766-3</t>
+          <t>130</t>
         </is>
       </c>
       <c r="B121" s="3" t="inlineStr">
@@ -13995,7 +13995,7 @@
       <c r="AR121" s="3" t="inlineStr"/>
       <c r="AS121" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18766-3</t>
+          <t>https://mia.nadimfoundation.org/130</t>
         </is>
       </c>
       <c r="AT121" s="3">
@@ -14036,7 +14036,7 @@
     <row r="122">
       <c r="A122" s="3" t="inlineStr">
         <is>
-          <t>18860-2</t>
+          <t>131</t>
         </is>
       </c>
       <c r="B122" s="3" t="inlineStr">
@@ -14112,7 +14112,7 @@
       <c r="AR122" s="3" t="inlineStr"/>
       <c r="AS122" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18860-2</t>
+          <t>https://mia.nadimfoundation.org/131</t>
         </is>
       </c>
       <c r="AT122" s="3">
@@ -14153,7 +14153,7 @@
     <row r="123">
       <c r="A123" s="3" t="inlineStr">
         <is>
-          <t>18860-5</t>
+          <t>132</t>
         </is>
       </c>
       <c r="B123" s="3" t="inlineStr">
@@ -14229,7 +14229,7 @@
       <c r="AR123" s="3" t="inlineStr"/>
       <c r="AS123" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18860-5</t>
+          <t>https://mia.nadimfoundation.org/132</t>
         </is>
       </c>
       <c r="AT123" s="3">
@@ -14270,7 +14270,7 @@
     <row r="124">
       <c r="A124" s="3" t="inlineStr">
         <is>
-          <t>18860-6</t>
+          <t>133</t>
         </is>
       </c>
       <c r="B124" s="3" t="inlineStr">
@@ -14346,7 +14346,7 @@
       <c r="AR124" s="3" t="inlineStr"/>
       <c r="AS124" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18860-6</t>
+          <t>https://mia.nadimfoundation.org/133</t>
         </is>
       </c>
       <c r="AT124" s="3">
@@ -14387,7 +14387,7 @@
     <row r="125">
       <c r="A125" s="3" t="inlineStr">
         <is>
-          <t>18860-7</t>
+          <t>134</t>
         </is>
       </c>
       <c r="B125" s="3" t="inlineStr">
@@ -14463,7 +14463,7 @@
       <c r="AR125" s="3" t="inlineStr"/>
       <c r="AS125" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18860-7</t>
+          <t>https://mia.nadimfoundation.org/134</t>
         </is>
       </c>
       <c r="AT125" s="3">
@@ -14504,7 +14504,7 @@
     <row r="126">
       <c r="A126" s="3" t="inlineStr">
         <is>
-          <t>3867</t>
+          <t>73</t>
         </is>
       </c>
       <c r="B126" s="3" t="inlineStr">
@@ -14580,7 +14580,7 @@
       <c r="AR126" s="3" t="inlineStr"/>
       <c r="AS126" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q3867</t>
+          <t>https://mia.nadimfoundation.org/73</t>
         </is>
       </c>
       <c r="AT126" s="3">
@@ -14601,7 +14601,7 @@
     <row r="127">
       <c r="A127" s="3" t="inlineStr">
         <is>
-          <t>4938</t>
+          <t>135</t>
         </is>
       </c>
       <c r="B127" s="3" t="inlineStr">
@@ -14685,7 +14685,7 @@
       <c r="AR127" s="3" t="inlineStr"/>
       <c r="AS127" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4938</t>
+          <t>https://mia.nadimfoundation.org/135</t>
         </is>
       </c>
       <c r="AT127" s="3">
@@ -14710,7 +14710,7 @@
     <row r="128">
       <c r="A128" s="3" t="inlineStr">
         <is>
-          <t>4939</t>
+          <t>136</t>
         </is>
       </c>
       <c r="B128" s="3" t="inlineStr">
@@ -14794,7 +14794,7 @@
       <c r="AR128" s="3" t="inlineStr"/>
       <c r="AS128" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4939</t>
+          <t>https://mia.nadimfoundation.org/136</t>
         </is>
       </c>
       <c r="AT128" s="3">
@@ -14819,7 +14819,7 @@
     <row r="129">
       <c r="A129" s="3" t="inlineStr">
         <is>
-          <t>4941</t>
+          <t>137</t>
         </is>
       </c>
       <c r="B129" s="3" t="inlineStr">
@@ -14903,7 +14903,7 @@
       <c r="AR129" s="3" t="inlineStr"/>
       <c r="AS129" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4941</t>
+          <t>https://mia.nadimfoundation.org/137</t>
         </is>
       </c>
       <c r="AT129" s="3">
@@ -14928,7 +14928,7 @@
     <row r="130">
       <c r="A130" s="3" t="inlineStr">
         <is>
-          <t>4942</t>
+          <t>138</t>
         </is>
       </c>
       <c r="B130" s="3" t="inlineStr">
@@ -15012,7 +15012,7 @@
       <c r="AR130" s="3" t="inlineStr"/>
       <c r="AS130" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4942</t>
+          <t>https://mia.nadimfoundation.org/138</t>
         </is>
       </c>
       <c r="AT130" s="3">
@@ -15037,7 +15037,7 @@
     <row r="131">
       <c r="A131" s="3" t="inlineStr">
         <is>
-          <t>4946</t>
+          <t>139</t>
         </is>
       </c>
       <c r="B131" s="3" t="inlineStr">
@@ -15121,7 +15121,7 @@
       <c r="AR131" s="3" t="inlineStr"/>
       <c r="AS131" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4946</t>
+          <t>https://mia.nadimfoundation.org/139</t>
         </is>
       </c>
       <c r="AT131" s="3">
@@ -15142,7 +15142,7 @@
     <row r="132">
       <c r="A132" s="3" t="inlineStr">
         <is>
-          <t>6621-1</t>
+          <t>140</t>
         </is>
       </c>
       <c r="B132" s="3" t="inlineStr">
@@ -15218,7 +15218,7 @@
       <c r="AR132" s="3" t="inlineStr"/>
       <c r="AS132" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q6621-1</t>
+          <t>https://mia.nadimfoundation.org/140</t>
         </is>
       </c>
       <c r="AT132" s="3">
@@ -15255,7 +15255,7 @@
     <row r="133">
       <c r="A133" s="3" t="inlineStr">
         <is>
-          <t>7936-1</t>
+          <t>141</t>
         </is>
       </c>
       <c r="B133" s="3" t="inlineStr">
@@ -15331,7 +15331,7 @@
       <c r="AR133" s="3" t="inlineStr"/>
       <c r="AS133" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q7936-1</t>
+          <t>https://mia.nadimfoundation.org/141</t>
         </is>
       </c>
       <c r="AT133" s="3">
@@ -15372,7 +15372,7 @@
     <row r="134">
       <c r="A134" s="3" t="inlineStr">
         <is>
-          <t>7936-4</t>
+          <t>142</t>
         </is>
       </c>
       <c r="B134" s="3" t="inlineStr">
@@ -15448,7 +15448,7 @@
       <c r="AR134" s="3" t="inlineStr"/>
       <c r="AS134" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q7936-4</t>
+          <t>https://mia.nadimfoundation.org/142</t>
         </is>
       </c>
       <c r="AT134" s="3">
@@ -15489,7 +15489,7 @@
     <row r="135">
       <c r="A135" s="3" t="inlineStr">
         <is>
-          <t>18761-1</t>
+          <t>143</t>
         </is>
       </c>
       <c r="B135" s="3" t="inlineStr">
@@ -15565,7 +15565,7 @@
       <c r="AR135" s="3" t="inlineStr"/>
       <c r="AS135" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18761-1</t>
+          <t>https://mia.nadimfoundation.org/143</t>
         </is>
       </c>
       <c r="AT135" s="3">
@@ -15606,7 +15606,7 @@
     <row r="136">
       <c r="A136" s="3" t="inlineStr">
         <is>
-          <t>18761-2</t>
+          <t>144</t>
         </is>
       </c>
       <c r="B136" s="3" t="inlineStr">
@@ -15682,7 +15682,7 @@
       <c r="AR136" s="3" t="inlineStr"/>
       <c r="AS136" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18761-2</t>
+          <t>https://mia.nadimfoundation.org/144</t>
         </is>
       </c>
       <c r="AT136" s="3">
@@ -15723,7 +15723,7 @@
     <row r="137">
       <c r="A137" s="3" t="inlineStr">
         <is>
-          <t>18761-3</t>
+          <t>145</t>
         </is>
       </c>
       <c r="B137" s="3" t="inlineStr">
@@ -15799,7 +15799,7 @@
       <c r="AR137" s="3" t="inlineStr"/>
       <c r="AS137" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18761-3</t>
+          <t>https://mia.nadimfoundation.org/145</t>
         </is>
       </c>
       <c r="AT137" s="3">
@@ -15840,7 +15840,7 @@
     <row r="138">
       <c r="A138" s="3" t="inlineStr">
         <is>
-          <t>18761-4</t>
+          <t>146</t>
         </is>
       </c>
       <c r="B138" s="3" t="inlineStr">
@@ -15916,7 +15916,7 @@
       <c r="AR138" s="3" t="inlineStr"/>
       <c r="AS138" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18761-4</t>
+          <t>https://mia.nadimfoundation.org/146</t>
         </is>
       </c>
       <c r="AT138" s="3">
@@ -15957,7 +15957,7 @@
     <row r="139">
       <c r="A139" s="3" t="inlineStr">
         <is>
-          <t>18761-5</t>
+          <t>147</t>
         </is>
       </c>
       <c r="B139" s="3" t="inlineStr">
@@ -16033,7 +16033,7 @@
       <c r="AR139" s="3" t="inlineStr"/>
       <c r="AS139" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18761-5</t>
+          <t>https://mia.nadimfoundation.org/147</t>
         </is>
       </c>
       <c r="AT139" s="3">
@@ -16074,7 +16074,7 @@
     <row r="140">
       <c r="A140" s="3" t="inlineStr">
         <is>
-          <t>18761-6</t>
+          <t>148</t>
         </is>
       </c>
       <c r="B140" s="3" t="inlineStr">
@@ -16150,7 +16150,7 @@
       <c r="AR140" s="3" t="inlineStr"/>
       <c r="AS140" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18761-6</t>
+          <t>https://mia.nadimfoundation.org/148</t>
         </is>
       </c>
       <c r="AT140" s="3">
@@ -16191,7 +16191,7 @@
     <row r="141">
       <c r="A141" s="3" t="inlineStr">
         <is>
-          <t>18761-7</t>
+          <t>149</t>
         </is>
       </c>
       <c r="B141" s="3" t="inlineStr">
@@ -16267,7 +16267,7 @@
       <c r="AR141" s="3" t="inlineStr"/>
       <c r="AS141" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18761-7</t>
+          <t>https://mia.nadimfoundation.org/149</t>
         </is>
       </c>
       <c r="AT141" s="3">
@@ -16308,7 +16308,7 @@
     <row r="142">
       <c r="A142" s="3" t="inlineStr">
         <is>
-          <t>18761-8</t>
+          <t>150</t>
         </is>
       </c>
       <c r="B142" s="3" t="inlineStr">
@@ -16384,7 +16384,7 @@
       <c r="AR142" s="3" t="inlineStr"/>
       <c r="AS142" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18761-8</t>
+          <t>https://mia.nadimfoundation.org/150</t>
         </is>
       </c>
       <c r="AT142" s="3">
@@ -16425,7 +16425,7 @@
     <row r="143">
       <c r="A143" s="3" t="inlineStr">
         <is>
-          <t>18761-9</t>
+          <t>151</t>
         </is>
       </c>
       <c r="B143" s="3" t="inlineStr">
@@ -16501,7 +16501,7 @@
       <c r="AR143" s="3" t="inlineStr"/>
       <c r="AS143" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18761-9</t>
+          <t>https://mia.nadimfoundation.org/151</t>
         </is>
       </c>
       <c r="AT143" s="3">
@@ -16542,7 +16542,7 @@
     <row r="144">
       <c r="A144" s="3" t="inlineStr">
         <is>
-          <t>18761-10</t>
+          <t>152</t>
         </is>
       </c>
       <c r="B144" s="3" t="inlineStr">
@@ -16618,7 +16618,7 @@
       <c r="AR144" s="3" t="inlineStr"/>
       <c r="AS144" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18761-10</t>
+          <t>https://mia.nadimfoundation.org/152</t>
         </is>
       </c>
       <c r="AT144" s="3">
@@ -16659,7 +16659,7 @@
     <row r="145">
       <c r="A145" s="3" t="inlineStr">
         <is>
-          <t>18761-11</t>
+          <t>153</t>
         </is>
       </c>
       <c r="B145" s="3" t="inlineStr">
@@ -16735,7 +16735,7 @@
       <c r="AR145" s="3" t="inlineStr"/>
       <c r="AS145" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18761-11</t>
+          <t>https://mia.nadimfoundation.org/153</t>
         </is>
       </c>
       <c r="AT145" s="3">
@@ -16776,7 +16776,7 @@
     <row r="146">
       <c r="A146" s="3" t="inlineStr">
         <is>
-          <t>18761-12</t>
+          <t>154</t>
         </is>
       </c>
       <c r="B146" s="3" t="inlineStr">
@@ -16852,7 +16852,7 @@
       <c r="AR146" s="3" t="inlineStr"/>
       <c r="AS146" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18761-12</t>
+          <t>https://mia.nadimfoundation.org/154</t>
         </is>
       </c>
       <c r="AT146" s="3">
@@ -16893,7 +16893,7 @@
     <row r="147">
       <c r="A147" s="3" t="inlineStr">
         <is>
-          <t>18761-13</t>
+          <t>155</t>
         </is>
       </c>
       <c r="B147" s="3" t="inlineStr">
@@ -16969,7 +16969,7 @@
       <c r="AR147" s="3" t="inlineStr"/>
       <c r="AS147" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18761-13</t>
+          <t>https://mia.nadimfoundation.org/155</t>
         </is>
       </c>
       <c r="AT147" s="3">
@@ -17010,7 +17010,7 @@
     <row r="148">
       <c r="A148" s="3" t="inlineStr">
         <is>
-          <t>18761-14</t>
+          <t>156</t>
         </is>
       </c>
       <c r="B148" s="3" t="inlineStr">
@@ -17086,7 +17086,7 @@
       <c r="AR148" s="3" t="inlineStr"/>
       <c r="AS148" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18761-14</t>
+          <t>https://mia.nadimfoundation.org/156</t>
         </is>
       </c>
       <c r="AT148" s="3">
@@ -17127,7 +17127,7 @@
     <row r="149">
       <c r="A149" s="3" t="inlineStr">
         <is>
-          <t>18761-15</t>
+          <t>157</t>
         </is>
       </c>
       <c r="B149" s="3" t="inlineStr">
@@ -17203,7 +17203,7 @@
       <c r="AR149" s="3" t="inlineStr"/>
       <c r="AS149" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18761-15</t>
+          <t>https://mia.nadimfoundation.org/157</t>
         </is>
       </c>
       <c r="AT149" s="3">
@@ -17244,7 +17244,7 @@
     <row r="150">
       <c r="A150" s="3" t="inlineStr">
         <is>
-          <t>18761-16</t>
+          <t>158</t>
         </is>
       </c>
       <c r="B150" s="3" t="inlineStr">
@@ -17320,7 +17320,7 @@
       <c r="AR150" s="3" t="inlineStr"/>
       <c r="AS150" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18761-16</t>
+          <t>https://mia.nadimfoundation.org/158</t>
         </is>
       </c>
       <c r="AT150" s="3">
@@ -17361,7 +17361,7 @@
     <row r="151">
       <c r="A151" s="3" t="inlineStr">
         <is>
-          <t>18761-17</t>
+          <t>159</t>
         </is>
       </c>
       <c r="B151" s="3" t="inlineStr">
@@ -17437,7 +17437,7 @@
       <c r="AR151" s="3" t="inlineStr"/>
       <c r="AS151" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18761-17</t>
+          <t>https://mia.nadimfoundation.org/159</t>
         </is>
       </c>
       <c r="AT151" s="3">
@@ -17478,7 +17478,7 @@
     <row r="152">
       <c r="A152" s="3" t="inlineStr">
         <is>
-          <t>18761-19</t>
+          <t>160</t>
         </is>
       </c>
       <c r="B152" s="3" t="inlineStr">
@@ -17554,7 +17554,7 @@
       <c r="AR152" s="3" t="inlineStr"/>
       <c r="AS152" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18761-19</t>
+          <t>https://mia.nadimfoundation.org/160</t>
         </is>
       </c>
       <c r="AT152" s="3">
@@ -17595,7 +17595,7 @@
     <row r="153">
       <c r="A153" s="3" t="inlineStr">
         <is>
-          <t>18761-20</t>
+          <t>161</t>
         </is>
       </c>
       <c r="B153" s="3" t="inlineStr">
@@ -17671,7 +17671,7 @@
       <c r="AR153" s="3" t="inlineStr"/>
       <c r="AS153" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18761-20</t>
+          <t>https://mia.nadimfoundation.org/161</t>
         </is>
       </c>
       <c r="AT153" s="3">
@@ -17712,7 +17712,7 @@
     <row r="154">
       <c r="A154" s="3" t="inlineStr">
         <is>
-          <t>18761-21</t>
+          <t>162</t>
         </is>
       </c>
       <c r="B154" s="3" t="inlineStr">
@@ -17788,7 +17788,7 @@
       <c r="AR154" s="3" t="inlineStr"/>
       <c r="AS154" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18761-21</t>
+          <t>https://mia.nadimfoundation.org/162</t>
         </is>
       </c>
       <c r="AT154" s="3">
@@ -17829,7 +17829,7 @@
     <row r="155">
       <c r="A155" s="3" t="inlineStr">
         <is>
-          <t>18761-22</t>
+          <t>163</t>
         </is>
       </c>
       <c r="B155" s="3" t="inlineStr">
@@ -17905,7 +17905,7 @@
       <c r="AR155" s="3" t="inlineStr"/>
       <c r="AS155" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18761-22</t>
+          <t>https://mia.nadimfoundation.org/163</t>
         </is>
       </c>
       <c r="AT155" s="3">
@@ -17946,7 +17946,7 @@
     <row r="156">
       <c r="A156" s="3" t="inlineStr">
         <is>
-          <t>18761-23</t>
+          <t>164</t>
         </is>
       </c>
       <c r="B156" s="3" t="inlineStr">
@@ -18022,7 +18022,7 @@
       <c r="AR156" s="3" t="inlineStr"/>
       <c r="AS156" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18761-23</t>
+          <t>https://mia.nadimfoundation.org/164</t>
         </is>
       </c>
       <c r="AT156" s="3">
@@ -18063,7 +18063,7 @@
     <row r="157">
       <c r="A157" s="3" t="inlineStr">
         <is>
-          <t>18761-24</t>
+          <t>165</t>
         </is>
       </c>
       <c r="B157" s="3" t="inlineStr">
@@ -18139,7 +18139,7 @@
       <c r="AR157" s="3" t="inlineStr"/>
       <c r="AS157" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18761-24</t>
+          <t>https://mia.nadimfoundation.org/165</t>
         </is>
       </c>
       <c r="AT157" s="3">
@@ -18180,7 +18180,7 @@
     <row r="158">
       <c r="A158" s="3" t="inlineStr">
         <is>
-          <t>4948</t>
+          <t>166</t>
         </is>
       </c>
       <c r="B158" s="3" t="inlineStr">
@@ -18264,7 +18264,7 @@
       <c r="AR158" s="3" t="inlineStr"/>
       <c r="AS158" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4948</t>
+          <t>https://mia.nadimfoundation.org/166</t>
         </is>
       </c>
       <c r="AT158" s="3">
@@ -18285,7 +18285,7 @@
     <row r="159">
       <c r="A159" s="3" t="inlineStr">
         <is>
-          <t>4949</t>
+          <t>167</t>
         </is>
       </c>
       <c r="B159" s="3" t="inlineStr">
@@ -18369,7 +18369,7 @@
       <c r="AR159" s="3" t="inlineStr"/>
       <c r="AS159" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4949</t>
+          <t>https://mia.nadimfoundation.org/167</t>
         </is>
       </c>
       <c r="AT159" s="3">
@@ -18390,7 +18390,7 @@
     <row r="160">
       <c r="A160" s="3" t="inlineStr">
         <is>
-          <t>4950</t>
+          <t>168</t>
         </is>
       </c>
       <c r="B160" s="3" t="inlineStr">
@@ -18474,7 +18474,7 @@
       <c r="AR160" s="3" t="inlineStr"/>
       <c r="AS160" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4950</t>
+          <t>https://mia.nadimfoundation.org/168</t>
         </is>
       </c>
       <c r="AT160" s="3">
@@ -18495,7 +18495,7 @@
     <row r="161">
       <c r="A161" s="3" t="inlineStr">
         <is>
-          <t>6120-2</t>
+          <t>169</t>
         </is>
       </c>
       <c r="B161" s="3" t="inlineStr">
@@ -18571,7 +18571,7 @@
       <c r="AR161" s="3" t="inlineStr"/>
       <c r="AS161" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q6120-2</t>
+          <t>https://mia.nadimfoundation.org/169</t>
         </is>
       </c>
       <c r="AT161" s="3">
@@ -18608,7 +18608,7 @@
     <row r="162">
       <c r="A162" s="3" t="inlineStr">
         <is>
-          <t>9015</t>
+          <t>170</t>
         </is>
       </c>
       <c r="B162" s="3" t="inlineStr">
@@ -18684,7 +18684,7 @@
       <c r="AR162" s="3" t="inlineStr"/>
       <c r="AS162" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q9015</t>
+          <t>https://mia.nadimfoundation.org/170</t>
         </is>
       </c>
       <c r="AT162" s="3">
@@ -18721,7 +18721,7 @@
     <row r="163">
       <c r="A163" s="3" t="inlineStr">
         <is>
-          <t>18765-8</t>
+          <t>171</t>
         </is>
       </c>
       <c r="B163" s="3" t="inlineStr">
@@ -18797,7 +18797,7 @@
       <c r="AR163" s="3" t="inlineStr"/>
       <c r="AS163" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18765-8</t>
+          <t>https://mia.nadimfoundation.org/171</t>
         </is>
       </c>
       <c r="AT163" s="3">
@@ -18834,7 +18834,7 @@
     <row r="164">
       <c r="A164" s="3" t="inlineStr">
         <is>
-          <t>4955</t>
+          <t>172</t>
         </is>
       </c>
       <c r="B164" s="3" t="inlineStr">
@@ -18918,7 +18918,7 @@
       <c r="AR164" s="3" t="inlineStr"/>
       <c r="AS164" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4955</t>
+          <t>https://mia.nadimfoundation.org/172</t>
         </is>
       </c>
       <c r="AT164" s="3">
@@ -18939,7 +18939,7 @@
     <row r="165">
       <c r="A165" s="3" t="inlineStr">
         <is>
-          <t>4956</t>
+          <t>173</t>
         </is>
       </c>
       <c r="B165" s="3" t="inlineStr">
@@ -19023,7 +19023,7 @@
       <c r="AR165" s="3" t="inlineStr"/>
       <c r="AS165" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4956</t>
+          <t>https://mia.nadimfoundation.org/173</t>
         </is>
       </c>
       <c r="AT165" s="3">
@@ -19044,7 +19044,7 @@
     <row r="166">
       <c r="A166" s="3" t="inlineStr">
         <is>
-          <t>4957</t>
+          <t>174</t>
         </is>
       </c>
       <c r="B166" s="3" t="inlineStr">
@@ -19128,7 +19128,7 @@
       <c r="AR166" s="3" t="inlineStr"/>
       <c r="AS166" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q4957</t>
+          <t>https://mia.nadimfoundation.org/174</t>
         </is>
       </c>
       <c r="AT166" s="3">
@@ -19149,7 +19149,7 @@
     <row r="167">
       <c r="A167" s="3" t="inlineStr">
         <is>
-          <t>18763-1</t>
+          <t>175</t>
         </is>
       </c>
       <c r="B167" s="3" t="inlineStr">
@@ -19225,7 +19225,7 @@
       <c r="AR167" s="3" t="inlineStr"/>
       <c r="AS167" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18763-1</t>
+          <t>https://mia.nadimfoundation.org/175</t>
         </is>
       </c>
       <c r="AT167" s="3">
@@ -19254,7 +19254,7 @@
     <row r="168">
       <c r="A168" s="3" t="inlineStr">
         <is>
-          <t>18763-2</t>
+          <t>176</t>
         </is>
       </c>
       <c r="B168" s="3" t="inlineStr">
@@ -19330,7 +19330,7 @@
       <c r="AR168" s="3" t="inlineStr"/>
       <c r="AS168" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q18763-2</t>
+          <t>https://mia.nadimfoundation.org/176</t>
         </is>
       </c>
       <c r="AT168" s="3">
@@ -19359,7 +19359,7 @@
     <row r="169">
       <c r="A169" s="3" t="inlineStr">
         <is>
-          <t>37773</t>
+          <t>76</t>
         </is>
       </c>
       <c r="B169" s="3" t="inlineStr">
@@ -19443,7 +19443,7 @@
       <c r="AR169" s="3" t="inlineStr"/>
       <c r="AS169" s="3" t="inlineStr">
         <is>
-          <t>https://mia.nadimfoundation.org/q37773</t>
+          <t>https://mia.nadimfoundation.org/76</t>
         </is>
       </c>
       <c r="AT169" s="3">

</xml_diff>